<commit_message>
Phase 1: audit closure report; record-number legacy rows; fix DC speed split
Closes (each proven by a check in scripts/build-data/audit-closure.mjs): fix audit #1-#2, #5-#19, #57, #81, #85, #102, #104, #107, #118-#129, #131, #144-#147, #150-#151, #156-#157, #162-#199, #263-#283, #302-#329, #339-#341

134 Fixed, 120 Tracked (data cannot be invented, rows stay draft), 94 Open. Only High issue still open: #4.
Legacy rows now use the audit's spreadsheet record numbering (multi-line cells in switching.csv).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/catalog/datacenter.xlsx
+++ b/data/catalog/datacenter.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2211" uniqueCount="751">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2211" uniqueCount="750">
   <si>
     <t>family</t>
   </si>
@@ -1391,10 +1391,7 @@
     <t>N9K-C9348GC-FX3</t>
   </si>
   <si>
-    <t>0.01, 0.1, 1</t>
-  </si>
-  <si>
-    <t>1, 10, 25, 40, 100</t>
+    <t>0.01, 0.1, 1, 10, 25</t>
   </si>
   <si>
     <t>DC-data.csv row 37</t>
@@ -1406,7 +1403,7 @@
     <t>N9K-C9348GC-FX3PH</t>
   </si>
   <si>
-    <t>0.1, 1</t>
+    <t>0.1, 1, 10, 25</t>
   </si>
   <si>
     <t>DC-data.csv row 38</t>
@@ -6754,7 +6751,7 @@
         <v>458</v>
       </c>
       <c r="AH37" t="s">
-        <v>459</v>
+        <v>374</v>
       </c>
       <c r="AJ37">
         <v>696</v>
@@ -6766,10 +6763,10 @@
         <v>351</v>
       </c>
       <c r="AM37" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="AN37" s="1" t="s">
         <v>460</v>
-      </c>
-      <c r="AN37" s="1" t="s">
-        <v>461</v>
       </c>
       <c r="AO37" s="1"/>
       <c r="AP37" s="1" t="s">
@@ -6781,7 +6778,7 @@
     </row>
     <row r="38" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B38" t="s">
         <v>97</v>
@@ -6796,10 +6793,10 @@
         <v>28</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
@@ -6834,10 +6831,10 @@
         <v>1</v>
       </c>
       <c r="AG38" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="AH38" t="s">
-        <v>459</v>
+        <v>374</v>
       </c>
       <c r="AJ38">
         <v>696</v>
@@ -6849,14 +6846,14 @@
         <v>351</v>
       </c>
       <c r="AM38" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="AN38" s="1" t="s">
         <v>464</v>
-      </c>
-      <c r="AN38" s="1" t="s">
-        <v>465</v>
       </c>
       <c r="AO38" s="1"/>
       <c r="AP38" s="1" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="AQ38" s="1" t="s">
         <v>3</v>
@@ -6864,13 +6861,13 @@
     </row>
     <row r="39" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="B39" t="s">
         <v>97</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="D39" t="s">
         <v>27</v>
@@ -6879,10 +6876,10 @@
         <v>28</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="H39" s="1"/>
       <c r="I39" s="1"/>
@@ -6900,7 +6897,7 @@
       <c r="U39" s="1"/>
       <c r="V39" s="1"/>
       <c r="W39" s="1" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="X39" s="1"/>
       <c r="Y39" s="1"/>
@@ -6932,10 +6929,10 @@
         <v>351</v>
       </c>
       <c r="AM39" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="AN39" s="1" t="s">
         <v>470</v>
-      </c>
-      <c r="AN39" s="1" t="s">
-        <v>471</v>
       </c>
       <c r="AO39" s="1"/>
       <c r="AP39" s="1" t="s">
@@ -6947,13 +6944,13 @@
     </row>
     <row r="40" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B40" t="s">
         <v>97</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="D40" t="s">
         <v>27</v>
@@ -6962,10 +6959,10 @@
         <v>28</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="H40" s="1"/>
       <c r="I40" s="1"/>
@@ -6983,7 +6980,7 @@
       <c r="U40" s="1"/>
       <c r="V40" s="1"/>
       <c r="W40" s="1" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="X40" s="1"/>
       <c r="Y40" s="1"/>
@@ -7015,10 +7012,10 @@
         <v>351</v>
       </c>
       <c r="AM40" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="AN40" s="1" t="s">
         <v>473</v>
-      </c>
-      <c r="AN40" s="1" t="s">
-        <v>474</v>
       </c>
       <c r="AO40" s="1"/>
       <c r="AP40" s="1" t="s">
@@ -7030,13 +7027,13 @@
     </row>
     <row r="41" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="B41" t="s">
         <v>97</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="D41" t="s">
         <v>27</v>
@@ -7045,10 +7042,10 @@
         <v>28</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="H41" s="1"/>
       <c r="I41" s="1"/>
@@ -7066,7 +7063,7 @@
       <c r="U41" s="1"/>
       <c r="V41" s="1"/>
       <c r="W41" s="1" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="X41" s="1"/>
       <c r="Y41" s="1"/>
@@ -7083,7 +7080,7 @@
         <v>2</v>
       </c>
       <c r="AG41" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="AH41" t="s">
         <v>374</v>
@@ -7098,10 +7095,10 @@
         <v>351</v>
       </c>
       <c r="AM41" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="AN41" s="1" t="s">
         <v>477</v>
-      </c>
-      <c r="AN41" s="1" t="s">
-        <v>478</v>
       </c>
       <c r="AO41" s="1"/>
       <c r="AP41" s="1" t="s">
@@ -7113,13 +7110,13 @@
     </row>
     <row r="42" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B42" t="s">
         <v>97</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="D42" t="s">
         <v>27</v>
@@ -7128,10 +7125,10 @@
         <v>28</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="H42" s="1"/>
       <c r="I42" s="1"/>
@@ -7149,7 +7146,7 @@
       <c r="U42" s="1"/>
       <c r="V42" s="1"/>
       <c r="W42" s="1" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="X42" s="1"/>
       <c r="Y42" s="1"/>
@@ -7166,7 +7163,7 @@
         <v>1.2</v>
       </c>
       <c r="AG42" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="AH42" t="s">
         <v>374</v>
@@ -7181,10 +7178,10 @@
         <v>351</v>
       </c>
       <c r="AM42" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="AN42" s="1" t="s">
         <v>480</v>
-      </c>
-      <c r="AN42" s="1" t="s">
-        <v>481</v>
       </c>
       <c r="AO42" s="1"/>
       <c r="AP42" s="1" t="s">
@@ -7196,13 +7193,13 @@
     </row>
     <row r="43" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B43" t="s">
         <v>97</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="D43" t="s">
         <v>27</v>
@@ -7211,10 +7208,10 @@
         <v>28</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="H43" s="1"/>
       <c r="I43" s="1"/>
@@ -7232,7 +7229,7 @@
       <c r="U43" s="1"/>
       <c r="V43" s="1"/>
       <c r="W43" s="1" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="X43" s="1"/>
       <c r="Y43" s="1"/>
@@ -7264,10 +7261,10 @@
         <v>289</v>
       </c>
       <c r="AM43" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="AN43" s="1" t="s">
         <v>483</v>
-      </c>
-      <c r="AN43" s="1" t="s">
-        <v>484</v>
       </c>
       <c r="AO43" s="1"/>
       <c r="AP43" s="1" t="s">
@@ -7279,13 +7276,13 @@
     </row>
     <row r="44" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B44" t="s">
         <v>97</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="D44" t="s">
         <v>27</v>
@@ -7294,10 +7291,10 @@
         <v>28</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="H44" s="1"/>
       <c r="I44" s="1"/>
@@ -7315,7 +7312,7 @@
       <c r="U44" s="1"/>
       <c r="V44" s="1"/>
       <c r="W44" s="1" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="X44" s="1"/>
       <c r="Y44" s="1"/>
@@ -7332,10 +7329,10 @@
         <v>1</v>
       </c>
       <c r="AG44" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="AH44" t="s">
-        <v>459</v>
+        <v>374</v>
       </c>
       <c r="AJ44">
         <v>696</v>
@@ -7344,17 +7341,17 @@
         <v>46</v>
       </c>
       <c r="AL44" t="s">
+        <v>487</v>
+      </c>
+      <c r="AM44" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="AM44" s="1" t="s">
+      <c r="AN44" s="1" t="s">
         <v>489</v>
-      </c>
-      <c r="AN44" s="1" t="s">
-        <v>490</v>
       </c>
       <c r="AO44" s="1"/>
       <c r="AP44" s="1" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="AQ44" s="1" t="s">
         <v>3</v>
@@ -7362,13 +7359,13 @@
     </row>
     <row r="45" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B45" t="s">
         <v>97</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="D45" t="s">
         <v>27</v>
@@ -7377,10 +7374,10 @@
         <v>28</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="H45" s="1"/>
       <c r="I45" s="1"/>
@@ -7391,17 +7388,17 @@
       </c>
       <c r="M45" s="1"/>
       <c r="N45" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="O45" s="1" t="s">
         <v>494</v>
-      </c>
-      <c r="O45" s="1" t="s">
-        <v>495</v>
       </c>
       <c r="P45" s="1" t="s">
         <v>373</v>
       </c>
       <c r="Q45" s="1"/>
       <c r="S45" s="1" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="T45" t="s">
         <v>108</v>
@@ -7409,7 +7406,7 @@
       <c r="U45" s="1"/>
       <c r="V45" s="1"/>
       <c r="W45" s="1" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="X45" s="1"/>
       <c r="Y45" s="1"/>
@@ -7441,10 +7438,10 @@
         <v>314</v>
       </c>
       <c r="AM45" s="1" t="s">
+        <v>497</v>
+      </c>
+      <c r="AN45" s="1" t="s">
         <v>498</v>
-      </c>
-      <c r="AN45" s="1" t="s">
-        <v>499</v>
       </c>
       <c r="AO45" s="1"/>
       <c r="AP45" s="1" t="s">
@@ -7454,13 +7451,13 @@
     </row>
     <row r="46" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="B46" t="s">
         <v>97</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="D46" t="s">
         <v>27</v>
@@ -7469,10 +7466,10 @@
         <v>28</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="H46" s="1"/>
       <c r="I46" s="1"/>
@@ -7490,7 +7487,7 @@
       <c r="U46" s="1"/>
       <c r="V46" s="1"/>
       <c r="W46" s="1" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="X46" s="1"/>
       <c r="Y46" s="1"/>
@@ -7522,14 +7519,14 @@
         <v>149</v>
       </c>
       <c r="AM46" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="AN46" s="1" t="s">
         <v>503</v>
-      </c>
-      <c r="AN46" s="1" t="s">
-        <v>504</v>
       </c>
       <c r="AO46" s="1"/>
       <c r="AP46" s="1" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="AQ46" s="1" t="s">
         <v>3</v>
@@ -7537,13 +7534,13 @@
     </row>
     <row r="47" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B47" t="s">
         <v>97</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="D47" t="s">
         <v>27</v>
@@ -7552,10 +7549,10 @@
         <v>28</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="H47" s="1"/>
       <c r="I47" s="1"/>
@@ -7570,7 +7567,7 @@
       <c r="P47" s="1"/>
       <c r="Q47" s="1"/>
       <c r="S47" s="1" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="T47" t="s">
         <v>108</v>
@@ -7578,7 +7575,7 @@
       <c r="U47" s="1"/>
       <c r="V47" s="1"/>
       <c r="W47" s="1" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="X47" s="1"/>
       <c r="Y47" s="1"/>
@@ -7595,10 +7592,10 @@
         <v>1</v>
       </c>
       <c r="AG47" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="AH47" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="AJ47">
         <v>960</v>
@@ -7607,10 +7604,10 @@
         <v>46</v>
       </c>
       <c r="AM47" s="1" t="s">
+        <v>509</v>
+      </c>
+      <c r="AN47" s="1" t="s">
         <v>510</v>
-      </c>
-      <c r="AN47" s="1" t="s">
-        <v>511</v>
       </c>
       <c r="AO47" s="1"/>
       <c r="AP47" s="1"/>
@@ -7618,13 +7615,13 @@
     </row>
     <row r="48" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="B48" t="s">
         <v>97</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="D48" t="s">
         <v>27</v>
@@ -7633,10 +7630,10 @@
         <v>28</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="H48" s="1"/>
       <c r="I48" s="1"/>
@@ -7651,7 +7648,7 @@
       <c r="P48" s="1"/>
       <c r="Q48" s="1"/>
       <c r="S48" s="1" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="T48" t="s">
         <v>108</v>
@@ -7659,7 +7656,7 @@
       <c r="U48" s="1"/>
       <c r="V48" s="1"/>
       <c r="W48" s="1" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="X48" s="1"/>
       <c r="Y48" s="1"/>
@@ -7676,10 +7673,10 @@
         <v>1</v>
       </c>
       <c r="AG48" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="AH48" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="AJ48">
         <v>480</v>
@@ -7688,10 +7685,10 @@
         <v>46</v>
       </c>
       <c r="AM48" s="1" t="s">
+        <v>512</v>
+      </c>
+      <c r="AN48" s="1" t="s">
         <v>513</v>
-      </c>
-      <c r="AN48" s="1" t="s">
-        <v>514</v>
       </c>
       <c r="AO48" s="1"/>
       <c r="AP48" s="1"/>
@@ -7699,13 +7696,13 @@
     </row>
     <row r="49" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B49" t="s">
         <v>97</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="D49" t="s">
         <v>27</v>
@@ -7714,10 +7711,10 @@
         <v>28</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="H49" s="1"/>
       <c r="I49" s="1"/>
@@ -7735,7 +7732,7 @@
       <c r="U49" s="1"/>
       <c r="V49" s="1"/>
       <c r="W49" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="X49" s="1"/>
       <c r="Y49" s="1"/>
@@ -7752,10 +7749,10 @@
         <v>9</v>
       </c>
       <c r="AG49" t="s">
+        <v>518</v>
+      </c>
+      <c r="AH49" t="s">
         <v>519</v>
-      </c>
-      <c r="AH49" t="s">
-        <v>520</v>
       </c>
       <c r="AI49">
         <v>4</v>
@@ -7767,17 +7764,17 @@
         <v>92</v>
       </c>
       <c r="AL49" t="s">
+        <v>520</v>
+      </c>
+      <c r="AM49" s="1" t="s">
         <v>521</v>
       </c>
-      <c r="AM49" s="1" t="s">
+      <c r="AN49" s="1" t="s">
         <v>522</v>
-      </c>
-      <c r="AN49" s="1" t="s">
-        <v>523</v>
       </c>
       <c r="AO49" s="1"/>
       <c r="AP49" s="1" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="AQ49" s="1" t="s">
         <v>3</v>
@@ -7785,13 +7782,13 @@
     </row>
     <row r="50" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="B50" t="s">
         <v>97</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="D50" t="s">
         <v>27</v>
@@ -7800,10 +7797,10 @@
         <v>28</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H50" s="1"/>
       <c r="I50" s="1"/>
@@ -7821,7 +7818,7 @@
       <c r="U50" s="1"/>
       <c r="V50" s="1"/>
       <c r="W50" s="1" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="X50" s="1"/>
       <c r="Y50" s="1"/>
@@ -7838,10 +7835,10 @@
         <v>14</v>
       </c>
       <c r="AG50" t="s">
+        <v>518</v>
+      </c>
+      <c r="AH50" t="s">
         <v>519</v>
-      </c>
-      <c r="AH50" t="s">
-        <v>520</v>
       </c>
       <c r="AI50">
         <v>8</v>
@@ -7853,17 +7850,17 @@
         <v>92</v>
       </c>
       <c r="AL50" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="AM50" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="AN50" s="1" t="s">
         <v>528</v>
-      </c>
-      <c r="AN50" s="1" t="s">
-        <v>529</v>
       </c>
       <c r="AO50" s="1"/>
       <c r="AP50" s="1" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="AQ50" s="1" t="s">
         <v>3</v>
@@ -7871,13 +7868,13 @@
     </row>
     <row r="51" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B51" t="s">
         <v>97</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="D51" t="s">
         <v>27</v>
@@ -7886,10 +7883,10 @@
         <v>28</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H51" s="1"/>
       <c r="I51" s="1"/>
@@ -7907,7 +7904,7 @@
       <c r="U51" s="1"/>
       <c r="V51" s="1"/>
       <c r="W51" s="1" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="X51" s="1"/>
       <c r="Y51" s="1"/>
@@ -7924,10 +7921,10 @@
         <v>26</v>
       </c>
       <c r="AG51" t="s">
+        <v>518</v>
+      </c>
+      <c r="AH51" t="s">
         <v>519</v>
-      </c>
-      <c r="AH51" t="s">
-        <v>520</v>
       </c>
       <c r="AI51">
         <v>16</v>
@@ -7939,17 +7936,17 @@
         <v>92</v>
       </c>
       <c r="AL51" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="AM51" s="1" t="s">
+        <v>532</v>
+      </c>
+      <c r="AN51" s="1" t="s">
         <v>533</v>
-      </c>
-      <c r="AN51" s="1" t="s">
-        <v>534</v>
       </c>
       <c r="AO51" s="1"/>
       <c r="AP51" s="1" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="AQ51" s="1" t="s">
         <v>3</v>
@@ -7957,13 +7954,13 @@
     </row>
     <row r="52" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B52" t="s">
         <v>97</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="D52" t="s">
         <v>27</v>
@@ -7972,10 +7969,10 @@
         <v>28</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="H52" s="1"/>
       <c r="I52" s="1"/>
@@ -7993,7 +7990,7 @@
       <c r="U52" s="1"/>
       <c r="V52" s="1"/>
       <c r="W52" s="1" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="X52" s="1"/>
       <c r="Y52" s="1"/>
@@ -8010,26 +8007,26 @@
         <v>2</v>
       </c>
       <c r="AG52" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="AH52" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="AK52" t="s">
         <v>92</v>
       </c>
       <c r="AL52" t="s">
+        <v>539</v>
+      </c>
+      <c r="AM52" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="AM52" s="1" t="s">
+      <c r="AN52" s="1" t="s">
         <v>541</v>
-      </c>
-      <c r="AN52" s="1" t="s">
-        <v>542</v>
       </c>
       <c r="AO52" s="1"/>
       <c r="AP52" s="1" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="AQ52" s="1" t="s">
         <v>3</v>
@@ -8037,13 +8034,13 @@
     </row>
     <row r="53" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B53" t="s">
         <v>97</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="D53" t="s">
         <v>27</v>
@@ -8052,10 +8049,10 @@
         <v>28</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="H53" s="1"/>
       <c r="I53" s="1"/>
@@ -8073,7 +8070,7 @@
       <c r="U53" s="1"/>
       <c r="V53" s="1"/>
       <c r="W53" s="1" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="X53" s="1"/>
       <c r="Y53" s="1"/>
@@ -8090,26 +8087,26 @@
         <v>2</v>
       </c>
       <c r="AG53" t="s">
+        <v>546</v>
+      </c>
+      <c r="AH53" t="s">
         <v>547</v>
-      </c>
-      <c r="AH53" t="s">
-        <v>548</v>
       </c>
       <c r="AK53" t="s">
         <v>92</v>
       </c>
       <c r="AL53" t="s">
+        <v>548</v>
+      </c>
+      <c r="AM53" s="1" t="s">
         <v>549</v>
       </c>
-      <c r="AM53" s="1" t="s">
+      <c r="AN53" s="1" t="s">
         <v>550</v>
-      </c>
-      <c r="AN53" s="1" t="s">
-        <v>551</v>
       </c>
       <c r="AO53" s="1"/>
       <c r="AP53" s="1" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="AQ53" s="1" t="s">
         <v>3</v>
@@ -8117,13 +8114,13 @@
     </row>
     <row r="54" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="B54" t="s">
         <v>97</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="D54" t="s">
         <v>27</v>
@@ -8132,10 +8129,10 @@
         <v>28</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="H54" s="1"/>
       <c r="I54" s="1"/>
@@ -8153,7 +8150,7 @@
       <c r="U54" s="1"/>
       <c r="V54" s="1"/>
       <c r="W54" s="1" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="X54" s="1"/>
       <c r="Y54" s="1"/>
@@ -8170,26 +8167,26 @@
         <v>1</v>
       </c>
       <c r="AG54" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="AH54" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="AK54" t="s">
         <v>92</v>
       </c>
       <c r="AL54" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="AM54" s="1" t="s">
+        <v>556</v>
+      </c>
+      <c r="AN54" s="1" t="s">
         <v>557</v>
-      </c>
-      <c r="AN54" s="1" t="s">
-        <v>558</v>
       </c>
       <c r="AO54" s="1"/>
       <c r="AP54" s="1" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="AQ54" s="1" t="s">
         <v>3</v>
@@ -8197,13 +8194,13 @@
     </row>
     <row r="55" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="B55" t="s">
         <v>97</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="D55" t="s">
         <v>27</v>
@@ -8212,10 +8209,10 @@
         <v>28</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="H55" s="1"/>
       <c r="I55" s="1"/>
@@ -8233,7 +8230,7 @@
       <c r="U55" s="1"/>
       <c r="V55" s="1"/>
       <c r="W55" s="1" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="X55" s="1"/>
       <c r="Y55" s="1"/>
@@ -8250,26 +8247,26 @@
         <v>1</v>
       </c>
       <c r="AG55" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="AH55" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="AK55" t="s">
         <v>92</v>
       </c>
       <c r="AL55" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="AM55" s="1" t="s">
+        <v>561</v>
+      </c>
+      <c r="AN55" s="1" t="s">
         <v>562</v>
-      </c>
-      <c r="AN55" s="1" t="s">
-        <v>563</v>
       </c>
       <c r="AO55" s="1"/>
       <c r="AP55" s="1" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="AQ55" s="1" t="s">
         <v>3</v>
@@ -8277,13 +8274,13 @@
     </row>
     <row r="56" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="B56" t="s">
         <v>97</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="D56" t="s">
         <v>27</v>
@@ -8292,10 +8289,10 @@
         <v>28</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="H56" s="1"/>
       <c r="I56" s="1"/>
@@ -8313,7 +8310,7 @@
       <c r="U56" s="1"/>
       <c r="V56" s="1"/>
       <c r="W56" s="1" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="X56" s="1"/>
       <c r="Y56" s="1"/>
@@ -8330,26 +8327,26 @@
         <v>1</v>
       </c>
       <c r="AG56" t="s">
+        <v>546</v>
+      </c>
+      <c r="AH56" t="s">
         <v>547</v>
-      </c>
-      <c r="AH56" t="s">
-        <v>548</v>
       </c>
       <c r="AK56" t="s">
         <v>92</v>
       </c>
       <c r="AL56" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="AM56" s="1" t="s">
+        <v>566</v>
+      </c>
+      <c r="AN56" s="1" t="s">
         <v>567</v>
-      </c>
-      <c r="AN56" s="1" t="s">
-        <v>568</v>
       </c>
       <c r="AO56" s="1"/>
       <c r="AP56" s="1" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="AQ56" s="1" t="s">
         <v>3</v>
@@ -8357,13 +8354,13 @@
     </row>
     <row r="57" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B57" t="s">
         <v>97</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="D57" t="s">
         <v>27</v>
@@ -8372,10 +8369,10 @@
         <v>28</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="H57" s="1"/>
       <c r="I57" s="1"/>
@@ -8393,7 +8390,7 @@
       <c r="U57" s="1"/>
       <c r="V57" s="1"/>
       <c r="W57" s="1" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="X57" s="1"/>
       <c r="Y57" s="1"/>
@@ -8410,26 +8407,26 @@
         <v>1</v>
       </c>
       <c r="AG57" t="s">
+        <v>546</v>
+      </c>
+      <c r="AH57" t="s">
         <v>547</v>
-      </c>
-      <c r="AH57" t="s">
-        <v>548</v>
       </c>
       <c r="AK57" t="s">
         <v>92</v>
       </c>
       <c r="AL57" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="AM57" s="1" t="s">
+        <v>570</v>
+      </c>
+      <c r="AN57" s="1" t="s">
         <v>571</v>
-      </c>
-      <c r="AN57" s="1" t="s">
-        <v>572</v>
       </c>
       <c r="AO57" s="1"/>
       <c r="AP57" s="1" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="AQ57" s="1" t="s">
         <v>3</v>
@@ -8437,13 +8434,13 @@
     </row>
     <row r="58" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="B58" t="s">
         <v>97</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="D58" t="s">
         <v>27</v>
@@ -8452,10 +8449,10 @@
         <v>28</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="H58" s="1"/>
       <c r="I58" s="1"/>
@@ -8473,7 +8470,7 @@
       <c r="U58" s="1"/>
       <c r="V58" s="1"/>
       <c r="W58" s="1" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="X58" s="1"/>
       <c r="Y58" s="1"/>
@@ -8487,26 +8484,26 @@
         <v>1</v>
       </c>
       <c r="AG58" t="s">
+        <v>576</v>
+      </c>
+      <c r="AH58" t="s">
         <v>577</v>
-      </c>
-      <c r="AH58" t="s">
-        <v>578</v>
       </c>
       <c r="AK58" t="s">
         <v>92</v>
       </c>
       <c r="AL58" t="s">
+        <v>578</v>
+      </c>
+      <c r="AM58" s="1" t="s">
         <v>579</v>
       </c>
-      <c r="AM58" s="1" t="s">
+      <c r="AN58" s="1" t="s">
         <v>580</v>
-      </c>
-      <c r="AN58" s="1" t="s">
-        <v>581</v>
       </c>
       <c r="AO58" s="1"/>
       <c r="AP58" s="1" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="AQ58" s="1" t="s">
         <v>3</v>
@@ -8514,13 +8511,13 @@
     </row>
     <row r="59" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="B59" t="s">
         <v>97</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="D59" t="s">
         <v>27</v>
@@ -8529,10 +8526,10 @@
         <v>28</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="H59" s="1"/>
       <c r="I59" s="1"/>
@@ -8550,7 +8547,7 @@
       <c r="U59" s="1"/>
       <c r="V59" s="1"/>
       <c r="W59" s="1" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="X59" s="1"/>
       <c r="Y59" s="1"/>
@@ -8582,16 +8579,16 @@
         <v>50</v>
       </c>
       <c r="AM59" s="1" t="s">
+        <v>585</v>
+      </c>
+      <c r="AN59" s="1" t="s">
         <v>586</v>
       </c>
-      <c r="AN59" s="1" t="s">
+      <c r="AO59" s="1" t="s">
         <v>587</v>
       </c>
-      <c r="AO59" s="1" t="s">
+      <c r="AP59" s="1" t="s">
         <v>588</v>
-      </c>
-      <c r="AP59" s="1" t="s">
-        <v>589</v>
       </c>
       <c r="AQ59" s="1" t="s">
         <v>3</v>
@@ -8599,13 +8596,13 @@
     </row>
     <row r="60" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="B60" t="s">
         <v>97</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="D60" t="s">
         <v>27</v>
@@ -8614,10 +8611,10 @@
         <v>28</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="H60" s="1"/>
       <c r="I60" s="1"/>
@@ -8635,7 +8632,7 @@
       <c r="U60" s="1"/>
       <c r="V60" s="1"/>
       <c r="W60" s="1" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="X60" s="1"/>
       <c r="Y60" s="1"/>
@@ -8652,7 +8649,7 @@
         <v>1</v>
       </c>
       <c r="AG60" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="AH60" t="s">
         <v>276</v>
@@ -8667,16 +8664,16 @@
         <v>50</v>
       </c>
       <c r="AM60" s="1" t="s">
+        <v>591</v>
+      </c>
+      <c r="AN60" s="1" t="s">
         <v>592</v>
       </c>
-      <c r="AN60" s="1" t="s">
+      <c r="AO60" s="1" t="s">
         <v>593</v>
       </c>
-      <c r="AO60" s="1" t="s">
+      <c r="AP60" s="1" t="s">
         <v>594</v>
-      </c>
-      <c r="AP60" s="1" t="s">
-        <v>595</v>
       </c>
       <c r="AQ60" s="1" t="s">
         <v>3</v>
@@ -8684,13 +8681,13 @@
     </row>
     <row r="61" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B61" t="s">
         <v>97</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="D61" t="s">
         <v>27</v>
@@ -8699,10 +8696,10 @@
         <v>28</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="H61" s="1"/>
       <c r="I61" s="1"/>
@@ -8720,7 +8717,7 @@
       <c r="U61" s="1"/>
       <c r="V61" s="1"/>
       <c r="W61" s="1" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="X61" s="1"/>
       <c r="Y61" s="1"/>
@@ -8749,16 +8746,16 @@
         <v>103</v>
       </c>
       <c r="AM61" s="1" t="s">
+        <v>596</v>
+      </c>
+      <c r="AN61" s="1" t="s">
         <v>597</v>
       </c>
-      <c r="AN61" s="1" t="s">
+      <c r="AO61" s="1" t="s">
         <v>598</v>
       </c>
-      <c r="AO61" s="1" t="s">
+      <c r="AP61" s="1" t="s">
         <v>599</v>
-      </c>
-      <c r="AP61" s="1" t="s">
-        <v>600</v>
       </c>
       <c r="AQ61" s="1" t="s">
         <v>3</v>
@@ -8823,7 +8820,7 @@
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>1</v>
@@ -8838,10 +8835,10 @@
         <v>238</v>
       </c>
       <c r="H1" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>602</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>603</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>6</v>
@@ -8900,7 +8897,7 @@
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B2" t="s">
         <v>97</v>
@@ -8915,10 +8912,10 @@
         <v>28</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="H2">
         <v>36</v>
@@ -8937,20 +8934,20 @@
       <c r="U2" s="1"/>
       <c r="V2" s="1"/>
       <c r="W2" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="X2" s="1" t="s">
         <v>605</v>
-      </c>
-      <c r="X2" s="1" t="s">
-        <v>606</v>
       </c>
       <c r="Y2" s="1"/>
       <c r="Z2" s="1"/>
       <c r="AA2" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B3" t="s">
         <v>97</v>
@@ -8965,10 +8962,10 @@
         <v>28</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H3">
         <v>36</v>
@@ -8987,20 +8984,20 @@
       <c r="U3" s="1"/>
       <c r="V3" s="1"/>
       <c r="W3" s="1" t="s">
+        <v>608</v>
+      </c>
+      <c r="X3" s="1" t="s">
         <v>609</v>
-      </c>
-      <c r="X3" s="1" t="s">
-        <v>610</v>
       </c>
       <c r="Y3" s="1"/>
       <c r="Z3" s="1"/>
       <c r="AA3" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B4" t="s">
         <v>97</v>
@@ -9015,10 +9012,10 @@
         <v>28</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="H4">
         <v>14</v>
@@ -9037,20 +9034,20 @@
       <c r="U4" s="1"/>
       <c r="V4" s="1"/>
       <c r="W4" s="1" t="s">
+        <v>611</v>
+      </c>
+      <c r="X4" s="1" t="s">
         <v>612</v>
-      </c>
-      <c r="X4" s="1" t="s">
-        <v>613</v>
       </c>
       <c r="Y4" s="1"/>
       <c r="Z4" s="1"/>
       <c r="AA4" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B5" t="s">
         <v>97</v>
@@ -9065,10 +9062,10 @@
         <v>28</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
@@ -9081,20 +9078,20 @@
       <c r="U5" s="1"/>
       <c r="V5" s="1"/>
       <c r="W5" s="1" t="s">
+        <v>614</v>
+      </c>
+      <c r="X5" s="1" t="s">
         <v>615</v>
-      </c>
-      <c r="X5" s="1" t="s">
-        <v>616</v>
       </c>
       <c r="Y5" s="1"/>
       <c r="Z5" s="1"/>
       <c r="AA5" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="B6" t="s">
         <v>97</v>
@@ -9109,10 +9106,10 @@
         <v>28</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
@@ -9125,20 +9122,20 @@
       <c r="U6" s="1"/>
       <c r="V6" s="1"/>
       <c r="W6" s="1" t="s">
+        <v>617</v>
+      </c>
+      <c r="X6" s="1" t="s">
         <v>618</v>
-      </c>
-      <c r="X6" s="1" t="s">
-        <v>619</v>
       </c>
       <c r="Y6" s="1"/>
       <c r="Z6" s="1"/>
       <c r="AA6" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="B7" t="s">
         <v>97</v>
@@ -9153,10 +9150,10 @@
         <v>28</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
@@ -9169,20 +9166,20 @@
       <c r="U7" s="1"/>
       <c r="V7" s="1"/>
       <c r="W7" s="1" t="s">
+        <v>620</v>
+      </c>
+      <c r="X7" s="1" t="s">
         <v>621</v>
-      </c>
-      <c r="X7" s="1" t="s">
-        <v>622</v>
       </c>
       <c r="Y7" s="1"/>
       <c r="Z7" s="1"/>
       <c r="AA7" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B8" t="s">
         <v>97</v>
@@ -9197,10 +9194,10 @@
         <v>28</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
@@ -9213,20 +9210,20 @@
       <c r="U8" s="1"/>
       <c r="V8" s="1"/>
       <c r="W8" s="1" t="s">
+        <v>623</v>
+      </c>
+      <c r="X8" s="1" t="s">
         <v>624</v>
-      </c>
-      <c r="X8" s="1" t="s">
-        <v>625</v>
       </c>
       <c r="Y8" s="1"/>
       <c r="Z8" s="1"/>
       <c r="AA8" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B9" t="s">
         <v>97</v>
@@ -9241,10 +9238,10 @@
         <v>28</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="H9">
         <v>16</v>
@@ -9263,20 +9260,20 @@
       <c r="U9" s="1"/>
       <c r="V9" s="1"/>
       <c r="W9" s="1" t="s">
+        <v>626</v>
+      </c>
+      <c r="X9" s="1" t="s">
         <v>627</v>
-      </c>
-      <c r="X9" s="1" t="s">
-        <v>628</v>
       </c>
       <c r="Y9" s="1"/>
       <c r="Z9" s="1"/>
       <c r="AA9" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B10" t="s">
         <v>97</v>
@@ -9291,10 +9288,10 @@
         <v>28</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="H10">
         <v>36</v>
@@ -9313,20 +9310,20 @@
       <c r="U10" s="1"/>
       <c r="V10" s="1"/>
       <c r="W10" s="1" t="s">
+        <v>629</v>
+      </c>
+      <c r="X10" s="1" t="s">
         <v>630</v>
-      </c>
-      <c r="X10" s="1" t="s">
-        <v>631</v>
       </c>
       <c r="Y10" s="1"/>
       <c r="Z10" s="1"/>
       <c r="AA10" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B11" t="s">
         <v>97</v>
@@ -9341,10 +9338,10 @@
         <v>28</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="H11">
         <v>36</v>
@@ -9357,27 +9354,27 @@
       </c>
       <c r="L11" s="1"/>
       <c r="M11" s="1" t="s">
+        <v>632</v>
+      </c>
+      <c r="N11" s="1" t="s">
         <v>633</v>
       </c>
-      <c r="N11" s="1" t="s">
-        <v>634</v>
-      </c>
       <c r="O11" s="1" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="P11" s="1"/>
       <c r="R11" s="1" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="S11" s="1"/>
       <c r="T11" s="1"/>
       <c r="U11" s="1"/>
       <c r="V11" s="1"/>
       <c r="W11" s="1" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="X11" s="1" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="Y11" s="1"/>
       <c r="Z11" s="1"/>
@@ -9387,7 +9384,7 @@
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B12" t="s">
         <v>97</v>
@@ -9402,10 +9399,10 @@
         <v>28</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="H12">
         <v>32</v>
@@ -9418,30 +9415,30 @@
       </c>
       <c r="L12" s="1"/>
       <c r="M12" s="1" t="s">
+        <v>637</v>
+      </c>
+      <c r="N12" s="1" t="s">
         <v>638</v>
       </c>
-      <c r="N12" s="1" t="s">
-        <v>639</v>
-      </c>
       <c r="O12" s="1" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="P12" s="1"/>
       <c r="R12" s="1" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="S12" s="1"/>
       <c r="T12" s="1"/>
       <c r="U12" s="1"/>
       <c r="V12" s="1"/>
       <c r="W12" s="1" t="s">
+        <v>640</v>
+      </c>
+      <c r="X12" s="1" t="s">
         <v>641</v>
       </c>
-      <c r="X12" s="1" t="s">
+      <c r="Y12" s="1" t="s">
         <v>642</v>
-      </c>
-      <c r="Y12" s="1" t="s">
-        <v>643</v>
       </c>
       <c r="Z12" s="1"/>
       <c r="AA12" s="1" t="s">
@@ -9450,7 +9447,7 @@
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B13" t="s">
         <v>97</v>
@@ -9465,16 +9462,16 @@
         <v>28</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="H13">
         <v>48</v>
       </c>
       <c r="I13" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
@@ -9487,20 +9484,20 @@
       <c r="U13" s="1"/>
       <c r="V13" s="1"/>
       <c r="W13" s="1" t="s">
+        <v>645</v>
+      </c>
+      <c r="X13" s="1" t="s">
         <v>646</v>
-      </c>
-      <c r="X13" s="1" t="s">
-        <v>647</v>
       </c>
       <c r="Y13" s="1"/>
       <c r="Z13" s="1"/>
       <c r="AA13" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="B14" t="s">
         <v>97</v>
@@ -9515,16 +9512,16 @@
         <v>28</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="H14">
         <v>48</v>
       </c>
       <c r="I14" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
@@ -9537,20 +9534,20 @@
       <c r="U14" s="1"/>
       <c r="V14" s="1"/>
       <c r="W14" s="1" t="s">
+        <v>648</v>
+      </c>
+      <c r="X14" s="1" t="s">
         <v>649</v>
-      </c>
-      <c r="X14" s="1" t="s">
-        <v>650</v>
       </c>
       <c r="Y14" s="1"/>
       <c r="Z14" s="1"/>
       <c r="AA14" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="B15" t="s">
         <v>97</v>
@@ -9565,10 +9562,10 @@
         <v>28</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="H15">
         <v>24</v>
@@ -9587,20 +9584,20 @@
       <c r="U15" s="1"/>
       <c r="V15" s="1"/>
       <c r="W15" s="1" t="s">
+        <v>651</v>
+      </c>
+      <c r="X15" s="1" t="s">
         <v>652</v>
-      </c>
-      <c r="X15" s="1" t="s">
-        <v>653</v>
       </c>
       <c r="Y15" s="1"/>
       <c r="Z15" s="1"/>
       <c r="AA15" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="B16" t="s">
         <v>97</v>
@@ -9615,10 +9612,10 @@
         <v>28</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="H16">
         <v>36</v>
@@ -9637,20 +9634,20 @@
       <c r="U16" s="1"/>
       <c r="V16" s="1"/>
       <c r="W16" s="1" t="s">
+        <v>654</v>
+      </c>
+      <c r="X16" s="1" t="s">
         <v>655</v>
-      </c>
-      <c r="X16" s="1" t="s">
-        <v>656</v>
       </c>
       <c r="Y16" s="1"/>
       <c r="Z16" s="1"/>
       <c r="AA16" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B17" t="s">
         <v>97</v>
@@ -9665,10 +9662,10 @@
         <v>28</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="H17">
         <v>36</v>
@@ -9687,20 +9684,20 @@
       <c r="U17" s="1"/>
       <c r="V17" s="1"/>
       <c r="W17" s="1" t="s">
+        <v>657</v>
+      </c>
+      <c r="X17" s="1" t="s">
         <v>658</v>
-      </c>
-      <c r="X17" s="1" t="s">
-        <v>659</v>
       </c>
       <c r="Y17" s="1"/>
       <c r="Z17" s="1"/>
       <c r="AA17" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B18" t="s">
         <v>97</v>
@@ -9715,16 +9712,16 @@
         <v>28</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="H18">
         <v>36</v>
       </c>
       <c r="I18" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="L18" s="1"/>
       <c r="M18" s="1"/>
@@ -9737,20 +9734,20 @@
       <c r="U18" s="1"/>
       <c r="V18" s="1"/>
       <c r="W18" s="1" t="s">
+        <v>661</v>
+      </c>
+      <c r="X18" s="1" t="s">
         <v>662</v>
-      </c>
-      <c r="X18" s="1" t="s">
-        <v>663</v>
       </c>
       <c r="Y18" s="1"/>
       <c r="Z18" s="1"/>
       <c r="AA18" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B19" t="s">
         <v>97</v>
@@ -9765,10 +9762,10 @@
         <v>28</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="H19">
         <v>32</v>
@@ -9787,20 +9784,20 @@
       <c r="U19" s="1"/>
       <c r="V19" s="1"/>
       <c r="W19" s="1" t="s">
+        <v>664</v>
+      </c>
+      <c r="X19" s="1" t="s">
         <v>665</v>
-      </c>
-      <c r="X19" s="1" t="s">
-        <v>666</v>
       </c>
       <c r="Y19" s="1"/>
       <c r="Z19" s="1"/>
       <c r="AA19" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B20" t="s">
         <v>97</v>
@@ -9815,10 +9812,10 @@
         <v>28</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="L20" s="1"/>
       <c r="M20" s="1"/>
@@ -9831,20 +9828,20 @@
       <c r="U20" s="1"/>
       <c r="V20" s="1"/>
       <c r="W20" s="1" t="s">
+        <v>667</v>
+      </c>
+      <c r="X20" s="1" t="s">
         <v>668</v>
-      </c>
-      <c r="X20" s="1" t="s">
-        <v>669</v>
       </c>
       <c r="Y20" s="1"/>
       <c r="Z20" s="1"/>
       <c r="AA20" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="B21" t="s">
         <v>97</v>
@@ -9859,10 +9856,10 @@
         <v>28</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="L21" s="1"/>
       <c r="M21" s="1"/>
@@ -9875,20 +9872,20 @@
       <c r="U21" s="1"/>
       <c r="V21" s="1"/>
       <c r="W21" s="1" t="s">
+        <v>670</v>
+      </c>
+      <c r="X21" s="1" t="s">
         <v>671</v>
-      </c>
-      <c r="X21" s="1" t="s">
-        <v>672</v>
       </c>
       <c r="Y21" s="1"/>
       <c r="Z21" s="1"/>
       <c r="AA21" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B22" t="s">
         <v>97</v>
@@ -9903,10 +9900,10 @@
         <v>28</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="L22" s="1"/>
       <c r="M22" s="1"/>
@@ -9919,20 +9916,20 @@
       <c r="U22" s="1"/>
       <c r="V22" s="1"/>
       <c r="W22" s="1" t="s">
+        <v>673</v>
+      </c>
+      <c r="X22" s="1" t="s">
         <v>674</v>
-      </c>
-      <c r="X22" s="1" t="s">
-        <v>675</v>
       </c>
       <c r="Y22" s="1"/>
       <c r="Z22" s="1"/>
       <c r="AA22" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="B23" t="s">
         <v>97</v>
@@ -9947,10 +9944,10 @@
         <v>28</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="L23" s="1"/>
       <c r="M23" s="1"/>
@@ -9963,20 +9960,20 @@
       <c r="U23" s="1"/>
       <c r="V23" s="1"/>
       <c r="W23" s="1" t="s">
+        <v>676</v>
+      </c>
+      <c r="X23" s="1" t="s">
         <v>677</v>
-      </c>
-      <c r="X23" s="1" t="s">
-        <v>678</v>
       </c>
       <c r="Y23" s="1"/>
       <c r="Z23" s="1"/>
       <c r="AA23" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B24" t="s">
         <v>97</v>
@@ -9991,10 +9988,10 @@
         <v>28</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="L24" s="1"/>
       <c r="M24" s="1"/>
@@ -10007,20 +10004,20 @@
       <c r="U24" s="1"/>
       <c r="V24" s="1"/>
       <c r="W24" s="1" t="s">
+        <v>679</v>
+      </c>
+      <c r="X24" s="1" t="s">
         <v>680</v>
-      </c>
-      <c r="X24" s="1" t="s">
-        <v>681</v>
       </c>
       <c r="Y24" s="1"/>
       <c r="Z24" s="1"/>
       <c r="AA24" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="B25" t="s">
         <v>97</v>
@@ -10035,10 +10032,10 @@
         <v>28</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="L25" s="1"/>
       <c r="M25" s="1"/>
@@ -10051,20 +10048,20 @@
       <c r="U25" s="1"/>
       <c r="V25" s="1"/>
       <c r="W25" s="1" t="s">
+        <v>682</v>
+      </c>
+      <c r="X25" s="1" t="s">
         <v>683</v>
-      </c>
-      <c r="X25" s="1" t="s">
-        <v>684</v>
       </c>
       <c r="Y25" s="1"/>
       <c r="Z25" s="1"/>
       <c r="AA25" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="B26" t="s">
         <v>97</v>
@@ -10079,10 +10076,10 @@
         <v>28</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
@@ -10095,20 +10092,20 @@
       <c r="U26" s="1"/>
       <c r="V26" s="1"/>
       <c r="W26" s="1" t="s">
+        <v>685</v>
+      </c>
+      <c r="X26" s="1" t="s">
         <v>686</v>
-      </c>
-      <c r="X26" s="1" t="s">
-        <v>687</v>
       </c>
       <c r="Y26" s="1"/>
       <c r="Z26" s="1"/>
       <c r="AA26" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="27" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="B27" t="s">
         <v>97</v>
@@ -10123,10 +10120,10 @@
         <v>28</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
@@ -10139,20 +10136,20 @@
       <c r="U27" s="1"/>
       <c r="V27" s="1"/>
       <c r="W27" s="1" t="s">
+        <v>688</v>
+      </c>
+      <c r="X27" s="1" t="s">
         <v>689</v>
-      </c>
-      <c r="X27" s="1" t="s">
-        <v>690</v>
       </c>
       <c r="Y27" s="1"/>
       <c r="Z27" s="1"/>
       <c r="AA27" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="28" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="B28" t="s">
         <v>97</v>
@@ -10167,10 +10164,10 @@
         <v>28</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
@@ -10183,20 +10180,20 @@
       <c r="U28" s="1"/>
       <c r="V28" s="1"/>
       <c r="W28" s="1" t="s">
+        <v>691</v>
+      </c>
+      <c r="X28" s="1" t="s">
         <v>692</v>
-      </c>
-      <c r="X28" s="1" t="s">
-        <v>693</v>
       </c>
       <c r="Y28" s="1"/>
       <c r="Z28" s="1"/>
       <c r="AA28" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="29" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="B29" t="s">
         <v>97</v>
@@ -10211,10 +10208,10 @@
         <v>28</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
@@ -10227,20 +10224,20 @@
       <c r="U29" s="1"/>
       <c r="V29" s="1"/>
       <c r="W29" s="1" t="s">
+        <v>694</v>
+      </c>
+      <c r="X29" s="1" t="s">
         <v>695</v>
-      </c>
-      <c r="X29" s="1" t="s">
-        <v>696</v>
       </c>
       <c r="Y29" s="1"/>
       <c r="Z29" s="1"/>
       <c r="AA29" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="30" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="B30" t="s">
         <v>97</v>
@@ -10255,10 +10252,10 @@
         <v>28</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="H30">
         <v>8</v>
@@ -10277,20 +10274,20 @@
       <c r="U30" s="1"/>
       <c r="V30" s="1"/>
       <c r="W30" s="1" t="s">
+        <v>697</v>
+      </c>
+      <c r="X30" s="1" t="s">
         <v>698</v>
-      </c>
-      <c r="X30" s="1" t="s">
-        <v>699</v>
       </c>
       <c r="Y30" s="1"/>
       <c r="Z30" s="1"/>
       <c r="AA30" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="31" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="B31" t="s">
         <v>97</v>
@@ -10305,16 +10302,16 @@
         <v>28</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="H31">
         <v>16</v>
       </c>
       <c r="I31" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
@@ -10327,20 +10324,20 @@
       <c r="U31" s="1"/>
       <c r="V31" s="1"/>
       <c r="W31" s="1" t="s">
+        <v>701</v>
+      </c>
+      <c r="X31" s="1" t="s">
         <v>702</v>
-      </c>
-      <c r="X31" s="1" t="s">
-        <v>703</v>
       </c>
       <c r="Y31" s="1"/>
       <c r="Z31" s="1"/>
       <c r="AA31" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="32" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="B32" t="s">
         <v>97</v>
@@ -10355,16 +10352,16 @@
         <v>28</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="H32">
         <v>22</v>
       </c>
       <c r="I32" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
@@ -10377,20 +10374,20 @@
       <c r="U32" s="1"/>
       <c r="V32" s="1"/>
       <c r="W32" s="1" t="s">
+        <v>705</v>
+      </c>
+      <c r="X32" s="1" t="s">
         <v>706</v>
-      </c>
-      <c r="X32" s="1" t="s">
-        <v>707</v>
       </c>
       <c r="Y32" s="1"/>
       <c r="Z32" s="1"/>
       <c r="AA32" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="33" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B33" t="s">
         <v>97</v>
@@ -10405,16 +10402,16 @@
         <v>28</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="H33">
         <v>24</v>
       </c>
       <c r="I33" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="L33" s="1"/>
       <c r="M33" s="1"/>
@@ -10427,20 +10424,20 @@
       <c r="U33" s="1"/>
       <c r="V33" s="1"/>
       <c r="W33" s="1" t="s">
+        <v>709</v>
+      </c>
+      <c r="X33" s="1" t="s">
         <v>710</v>
-      </c>
-      <c r="X33" s="1" t="s">
-        <v>711</v>
       </c>
       <c r="Y33" s="1"/>
       <c r="Z33" s="1"/>
       <c r="AA33" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="34" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="B34" t="s">
         <v>97</v>
@@ -10455,16 +10452,16 @@
         <v>28</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="H34">
         <v>48</v>
       </c>
       <c r="I34" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="L34" s="1"/>
       <c r="M34" s="1"/>
@@ -10477,20 +10474,20 @@
       <c r="U34" s="1"/>
       <c r="V34" s="1"/>
       <c r="W34" s="1" t="s">
+        <v>712</v>
+      </c>
+      <c r="X34" s="1" t="s">
         <v>713</v>
-      </c>
-      <c r="X34" s="1" t="s">
-        <v>714</v>
       </c>
       <c r="Y34" s="1"/>
       <c r="Z34" s="1"/>
       <c r="AA34" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="35" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="B35" t="s">
         <v>97</v>
@@ -10505,16 +10502,16 @@
         <v>28</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="H35">
         <v>48</v>
       </c>
       <c r="I35" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="L35" s="1"/>
       <c r="M35" s="1"/>
@@ -10527,20 +10524,20 @@
       <c r="U35" s="1"/>
       <c r="V35" s="1"/>
       <c r="W35" s="1" t="s">
+        <v>715</v>
+      </c>
+      <c r="X35" s="1" t="s">
         <v>716</v>
-      </c>
-      <c r="X35" s="1" t="s">
-        <v>717</v>
       </c>
       <c r="Y35" s="1"/>
       <c r="Z35" s="1"/>
       <c r="AA35" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="36" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="B36" t="s">
         <v>97</v>
@@ -10555,16 +10552,16 @@
         <v>28</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="H36">
         <v>48</v>
       </c>
       <c r="I36" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
@@ -10577,20 +10574,20 @@
       <c r="U36" s="1"/>
       <c r="V36" s="1"/>
       <c r="W36" s="1" t="s">
+        <v>718</v>
+      </c>
+      <c r="X36" s="1" t="s">
         <v>719</v>
-      </c>
-      <c r="X36" s="1" t="s">
-        <v>720</v>
       </c>
       <c r="Y36" s="1"/>
       <c r="Z36" s="1"/>
       <c r="AA36" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="37" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="B37" t="s">
         <v>97</v>
@@ -10605,16 +10602,16 @@
         <v>28</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="H37">
         <v>48</v>
       </c>
       <c r="I37" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="L37" s="1"/>
       <c r="M37" s="1"/>
@@ -10627,20 +10624,20 @@
       <c r="U37" s="1"/>
       <c r="V37" s="1"/>
       <c r="W37" s="1" t="s">
+        <v>721</v>
+      </c>
+      <c r="X37" s="1" t="s">
         <v>722</v>
-      </c>
-      <c r="X37" s="1" t="s">
-        <v>723</v>
       </c>
       <c r="Y37" s="1"/>
       <c r="Z37" s="1"/>
       <c r="AA37" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="38" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="B38" t="s">
         <v>97</v>
@@ -10655,10 +10652,10 @@
         <v>28</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="L38" s="1"/>
       <c r="M38" s="1"/>
@@ -10671,20 +10668,20 @@
       <c r="U38" s="1"/>
       <c r="V38" s="1"/>
       <c r="W38" s="1" t="s">
+        <v>724</v>
+      </c>
+      <c r="X38" s="1" t="s">
         <v>725</v>
-      </c>
-      <c r="X38" s="1" t="s">
-        <v>726</v>
       </c>
       <c r="Y38" s="1"/>
       <c r="Z38" s="1"/>
       <c r="AA38" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="39" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="B39" t="s">
         <v>97</v>
@@ -10699,10 +10696,10 @@
         <v>28</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="L39" s="1"/>
       <c r="M39" s="1"/>
@@ -10715,20 +10712,20 @@
       <c r="U39" s="1"/>
       <c r="V39" s="1"/>
       <c r="W39" s="1" t="s">
+        <v>727</v>
+      </c>
+      <c r="X39" s="1" t="s">
         <v>728</v>
-      </c>
-      <c r="X39" s="1" t="s">
-        <v>729</v>
       </c>
       <c r="Y39" s="1"/>
       <c r="Z39" s="1"/>
       <c r="AA39" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="40" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="B40" t="s">
         <v>97</v>
@@ -10743,10 +10740,10 @@
         <v>28</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="L40" s="1"/>
       <c r="M40" s="1"/>
@@ -10759,15 +10756,15 @@
       <c r="U40" s="1"/>
       <c r="V40" s="1"/>
       <c r="W40" s="1" t="s">
+        <v>730</v>
+      </c>
+      <c r="X40" s="1" t="s">
         <v>731</v>
-      </c>
-      <c r="X40" s="1" t="s">
-        <v>732</v>
       </c>
       <c r="Y40" s="1"/>
       <c r="Z40" s="1"/>
       <c r="AA40" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
   </sheetData>
@@ -10808,827 +10805,827 @@
   <sheetData>
     <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>732</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>733</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>734</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>735</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>271</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>281</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>271</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>281</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>271</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>281</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>271</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>281</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>271</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>281</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>271</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>281</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>271</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>281</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>284</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>293</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>284</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>293</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>284</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>293</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>284</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>293</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>284</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>293</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>284</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>293</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>293</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>284</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>293</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>284</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>293</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>284</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>293</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>284</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>293</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>284</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>284</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>284</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>293</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>293</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>293</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>293</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>284</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>293</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>284</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="B54" s="1" t="s">
         <v>293</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="B55" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="B56" s="1" t="s">
         <v>299</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="B57" s="1" t="s">
         <v>299</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="B58" s="1" t="s">
         <v>299</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
     </row>
   </sheetData>
@@ -11663,10 +11660,10 @@
         <v>2</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>749</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>750</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -11674,7 +11671,7 @@
         <v>97</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="C2" t="s">
         <v>27</v>
@@ -11690,7 +11687,7 @@
         <v>97</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="C3" t="s">
         <v>27</v>
@@ -11706,7 +11703,7 @@
         <v>97</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="C4" t="s">
         <v>27</v>
@@ -11722,7 +11719,7 @@
         <v>97</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="C5" t="s">
         <v>27</v>
@@ -11738,7 +11735,7 @@
         <v>97</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="C6" t="s">
         <v>27</v>
@@ -11786,7 +11783,7 @@
         <v>97</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="C9" t="s">
         <v>27</v>
@@ -11834,7 +11831,7 @@
         <v>97</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="C12" t="s">
         <v>27</v>
@@ -11866,7 +11863,7 @@
         <v>97</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="C14" t="s">
         <v>27</v>
@@ -11994,7 +11991,7 @@
         <v>97</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="C22" t="s">
         <v>27</v>

</xml_diff>

<commit_message>
Phase 1: apply spec-reviewer findings
- audit #18/#19: end-of-sale network modules get replacement_none; switches keep the PID link
- current rows carry no end-of-sale bulletin; lifecycles from the legacy label or a third-party source are flagged per row
- inferred false values (ac_powered, poe, uplink_mgig) are now empty
- validator: BAD_PID (ready rows), SERIES_NOT_READY, NON_CISCO_SOURCE warning
- bare cisco.com links become https://www.cisco.com; closure wording made precise
- drop unused zod; migration tests no longer break when rows become ready

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/catalog/datacenter.xlsx
+++ b/data/catalog/datacenter.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2216" uniqueCount="756">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2214" uniqueCount="755">
   <si>
     <t>family</t>
   </si>
@@ -1548,9 +1548,6 @@
   </si>
   <si>
     <t>N3K-C3548P-XL</t>
-  </si>
-  <si>
-    <t>https://www.cisco.com/c/en/us/products/collateral/switches/nexus-3000-series-switches/nexus-3524-x-3548-x-eol.html</t>
   </si>
   <si>
     <t>https://www.cisco.com/c/en/us/products/collateral/switches/nexus-3548-switch/data_sheet_c78-707001.html</t>
@@ -7596,16 +7593,14 @@
       <c r="O47" s="1"/>
       <c r="P47" s="1"/>
       <c r="Q47" s="1"/>
-      <c r="S47" s="1" t="s">
-        <v>511</v>
-      </c>
+      <c r="S47" s="1"/>
       <c r="T47" t="s">
         <v>108</v>
       </c>
       <c r="U47" s="1"/>
       <c r="V47" s="1"/>
       <c r="W47" s="1" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="X47" s="1"/>
       <c r="Y47" s="1"/>
@@ -7622,10 +7617,10 @@
         <v>1</v>
       </c>
       <c r="AG47" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="AH47" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="AJ47">
         <v>960</v>
@@ -7634,10 +7629,10 @@
         <v>46</v>
       </c>
       <c r="AM47" s="1" t="s">
+        <v>513</v>
+      </c>
+      <c r="AN47" s="1" t="s">
         <v>514</v>
-      </c>
-      <c r="AN47" s="1" t="s">
-        <v>515</v>
       </c>
       <c r="AO47" s="1"/>
       <c r="AP47" s="1"/>
@@ -7645,7 +7640,7 @@
     </row>
     <row r="48" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="B48" t="s">
         <v>97</v>
@@ -7660,10 +7655,10 @@
         <v>28</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="H48" s="1"/>
       <c r="I48" s="1"/>
@@ -7677,16 +7672,14 @@
       <c r="O48" s="1"/>
       <c r="P48" s="1"/>
       <c r="Q48" s="1"/>
-      <c r="S48" s="1" t="s">
-        <v>511</v>
-      </c>
+      <c r="S48" s="1"/>
       <c r="T48" t="s">
         <v>108</v>
       </c>
       <c r="U48" s="1"/>
       <c r="V48" s="1"/>
       <c r="W48" s="1" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="X48" s="1"/>
       <c r="Y48" s="1"/>
@@ -7703,10 +7696,10 @@
         <v>1</v>
       </c>
       <c r="AG48" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="AH48" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="AJ48">
         <v>480</v>
@@ -7715,10 +7708,10 @@
         <v>46</v>
       </c>
       <c r="AM48" s="1" t="s">
+        <v>516</v>
+      </c>
+      <c r="AN48" s="1" t="s">
         <v>517</v>
-      </c>
-      <c r="AN48" s="1" t="s">
-        <v>518</v>
       </c>
       <c r="AO48" s="1"/>
       <c r="AP48" s="1"/>
@@ -7726,13 +7719,13 @@
     </row>
     <row r="49" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B49" t="s">
         <v>97</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="D49" t="s">
         <v>27</v>
@@ -7741,10 +7734,10 @@
         <v>28</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="H49" s="1"/>
       <c r="I49" s="1"/>
@@ -7762,7 +7755,7 @@
       <c r="U49" s="1"/>
       <c r="V49" s="1"/>
       <c r="W49" s="1" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="X49" s="1"/>
       <c r="Y49" s="1"/>
@@ -7779,10 +7772,10 @@
         <v>9</v>
       </c>
       <c r="AG49" t="s">
+        <v>522</v>
+      </c>
+      <c r="AH49" t="s">
         <v>523</v>
-      </c>
-      <c r="AH49" t="s">
-        <v>524</v>
       </c>
       <c r="AI49">
         <v>4</v>
@@ -7794,17 +7787,17 @@
         <v>92</v>
       </c>
       <c r="AL49" t="s">
+        <v>524</v>
+      </c>
+      <c r="AM49" s="1" t="s">
         <v>525</v>
       </c>
-      <c r="AM49" s="1" t="s">
+      <c r="AN49" s="1" t="s">
         <v>526</v>
-      </c>
-      <c r="AN49" s="1" t="s">
-        <v>527</v>
       </c>
       <c r="AO49" s="1"/>
       <c r="AP49" s="1" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="AQ49" s="1" t="s">
         <v>3</v>
@@ -7812,13 +7805,13 @@
     </row>
     <row r="50" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="B50" t="s">
         <v>97</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="D50" t="s">
         <v>27</v>
@@ -7827,10 +7820,10 @@
         <v>28</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="H50" s="1"/>
       <c r="I50" s="1"/>
@@ -7848,7 +7841,7 @@
       <c r="U50" s="1"/>
       <c r="V50" s="1"/>
       <c r="W50" s="1" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="X50" s="1"/>
       <c r="Y50" s="1"/>
@@ -7865,10 +7858,10 @@
         <v>14</v>
       </c>
       <c r="AG50" t="s">
+        <v>522</v>
+      </c>
+      <c r="AH50" t="s">
         <v>523</v>
-      </c>
-      <c r="AH50" t="s">
-        <v>524</v>
       </c>
       <c r="AI50">
         <v>8</v>
@@ -7880,17 +7873,17 @@
         <v>92</v>
       </c>
       <c r="AL50" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="AM50" s="1" t="s">
+        <v>531</v>
+      </c>
+      <c r="AN50" s="1" t="s">
         <v>532</v>
-      </c>
-      <c r="AN50" s="1" t="s">
-        <v>533</v>
       </c>
       <c r="AO50" s="1"/>
       <c r="AP50" s="1" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="AQ50" s="1" t="s">
         <v>3</v>
@@ -7898,13 +7891,13 @@
     </row>
     <row r="51" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B51" t="s">
         <v>97</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="D51" t="s">
         <v>27</v>
@@ -7913,10 +7906,10 @@
         <v>28</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="H51" s="1"/>
       <c r="I51" s="1"/>
@@ -7934,7 +7927,7 @@
       <c r="U51" s="1"/>
       <c r="V51" s="1"/>
       <c r="W51" s="1" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="X51" s="1"/>
       <c r="Y51" s="1"/>
@@ -7951,10 +7944,10 @@
         <v>26</v>
       </c>
       <c r="AG51" t="s">
+        <v>522</v>
+      </c>
+      <c r="AH51" t="s">
         <v>523</v>
-      </c>
-      <c r="AH51" t="s">
-        <v>524</v>
       </c>
       <c r="AI51">
         <v>16</v>
@@ -7966,17 +7959,17 @@
         <v>92</v>
       </c>
       <c r="AL51" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="AM51" s="1" t="s">
+        <v>536</v>
+      </c>
+      <c r="AN51" s="1" t="s">
         <v>537</v>
-      </c>
-      <c r="AN51" s="1" t="s">
-        <v>538</v>
       </c>
       <c r="AO51" s="1"/>
       <c r="AP51" s="1" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="AQ51" s="1" t="s">
         <v>3</v>
@@ -7984,13 +7977,13 @@
     </row>
     <row r="52" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="B52" t="s">
         <v>97</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="D52" t="s">
         <v>27</v>
@@ -7999,10 +7992,10 @@
         <v>28</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="H52" s="1"/>
       <c r="I52" s="1"/>
@@ -8020,7 +8013,7 @@
       <c r="U52" s="1"/>
       <c r="V52" s="1"/>
       <c r="W52" s="1" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="X52" s="1"/>
       <c r="Y52" s="1"/>
@@ -8037,26 +8030,26 @@
         <v>2</v>
       </c>
       <c r="AG52" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="AH52" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="AK52" t="s">
         <v>92</v>
       </c>
       <c r="AL52" t="s">
+        <v>543</v>
+      </c>
+      <c r="AM52" s="1" t="s">
         <v>544</v>
       </c>
-      <c r="AM52" s="1" t="s">
+      <c r="AN52" s="1" t="s">
         <v>545</v>
-      </c>
-      <c r="AN52" s="1" t="s">
-        <v>546</v>
       </c>
       <c r="AO52" s="1"/>
       <c r="AP52" s="1" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="AQ52" s="1" t="s">
         <v>3</v>
@@ -8064,13 +8057,13 @@
     </row>
     <row r="53" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B53" t="s">
         <v>97</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="D53" t="s">
         <v>27</v>
@@ -8079,10 +8072,10 @@
         <v>28</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="H53" s="1"/>
       <c r="I53" s="1"/>
@@ -8100,7 +8093,7 @@
       <c r="U53" s="1"/>
       <c r="V53" s="1"/>
       <c r="W53" s="1" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="X53" s="1"/>
       <c r="Y53" s="1"/>
@@ -8117,26 +8110,26 @@
         <v>2</v>
       </c>
       <c r="AG53" t="s">
+        <v>550</v>
+      </c>
+      <c r="AH53" t="s">
         <v>551</v>
-      </c>
-      <c r="AH53" t="s">
-        <v>552</v>
       </c>
       <c r="AK53" t="s">
         <v>92</v>
       </c>
       <c r="AL53" t="s">
+        <v>552</v>
+      </c>
+      <c r="AM53" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="AM53" s="1" t="s">
+      <c r="AN53" s="1" t="s">
         <v>554</v>
-      </c>
-      <c r="AN53" s="1" t="s">
-        <v>555</v>
       </c>
       <c r="AO53" s="1"/>
       <c r="AP53" s="1" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="AQ53" s="1" t="s">
         <v>3</v>
@@ -8144,13 +8137,13 @@
     </row>
     <row r="54" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="B54" t="s">
         <v>97</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="D54" t="s">
         <v>27</v>
@@ -8159,10 +8152,10 @@
         <v>28</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="H54" s="1"/>
       <c r="I54" s="1"/>
@@ -8180,7 +8173,7 @@
       <c r="U54" s="1"/>
       <c r="V54" s="1"/>
       <c r="W54" s="1" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="X54" s="1"/>
       <c r="Y54" s="1"/>
@@ -8197,26 +8190,26 @@
         <v>1</v>
       </c>
       <c r="AG54" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="AH54" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="AK54" t="s">
         <v>92</v>
       </c>
       <c r="AL54" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="AM54" s="1" t="s">
+        <v>560</v>
+      </c>
+      <c r="AN54" s="1" t="s">
         <v>561</v>
-      </c>
-      <c r="AN54" s="1" t="s">
-        <v>562</v>
       </c>
       <c r="AO54" s="1"/>
       <c r="AP54" s="1" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="AQ54" s="1" t="s">
         <v>3</v>
@@ -8224,13 +8217,13 @@
     </row>
     <row r="55" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="B55" t="s">
         <v>97</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="D55" t="s">
         <v>27</v>
@@ -8239,10 +8232,10 @@
         <v>28</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="H55" s="1"/>
       <c r="I55" s="1"/>
@@ -8260,7 +8253,7 @@
       <c r="U55" s="1"/>
       <c r="V55" s="1"/>
       <c r="W55" s="1" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="X55" s="1"/>
       <c r="Y55" s="1"/>
@@ -8277,26 +8270,26 @@
         <v>1</v>
       </c>
       <c r="AG55" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="AH55" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="AK55" t="s">
         <v>92</v>
       </c>
       <c r="AL55" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="AM55" s="1" t="s">
+        <v>565</v>
+      </c>
+      <c r="AN55" s="1" t="s">
         <v>566</v>
-      </c>
-      <c r="AN55" s="1" t="s">
-        <v>567</v>
       </c>
       <c r="AO55" s="1"/>
       <c r="AP55" s="1" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="AQ55" s="1" t="s">
         <v>3</v>
@@ -8304,13 +8297,13 @@
     </row>
     <row r="56" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="B56" t="s">
         <v>97</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="D56" t="s">
         <v>27</v>
@@ -8319,10 +8312,10 @@
         <v>28</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="H56" s="1"/>
       <c r="I56" s="1"/>
@@ -8340,7 +8333,7 @@
       <c r="U56" s="1"/>
       <c r="V56" s="1"/>
       <c r="W56" s="1" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="X56" s="1"/>
       <c r="Y56" s="1"/>
@@ -8357,26 +8350,26 @@
         <v>1</v>
       </c>
       <c r="AG56" t="s">
+        <v>550</v>
+      </c>
+      <c r="AH56" t="s">
         <v>551</v>
-      </c>
-      <c r="AH56" t="s">
-        <v>552</v>
       </c>
       <c r="AK56" t="s">
         <v>92</v>
       </c>
       <c r="AL56" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="AM56" s="1" t="s">
+        <v>570</v>
+      </c>
+      <c r="AN56" s="1" t="s">
         <v>571</v>
-      </c>
-      <c r="AN56" s="1" t="s">
-        <v>572</v>
       </c>
       <c r="AO56" s="1"/>
       <c r="AP56" s="1" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="AQ56" s="1" t="s">
         <v>3</v>
@@ -8384,13 +8377,13 @@
     </row>
     <row r="57" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="B57" t="s">
         <v>97</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="D57" t="s">
         <v>27</v>
@@ -8399,10 +8392,10 @@
         <v>28</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="H57" s="1"/>
       <c r="I57" s="1"/>
@@ -8420,7 +8413,7 @@
       <c r="U57" s="1"/>
       <c r="V57" s="1"/>
       <c r="W57" s="1" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="X57" s="1"/>
       <c r="Y57" s="1"/>
@@ -8437,26 +8430,26 @@
         <v>1</v>
       </c>
       <c r="AG57" t="s">
+        <v>550</v>
+      </c>
+      <c r="AH57" t="s">
         <v>551</v>
-      </c>
-      <c r="AH57" t="s">
-        <v>552</v>
       </c>
       <c r="AK57" t="s">
         <v>92</v>
       </c>
       <c r="AL57" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="AM57" s="1" t="s">
+        <v>574</v>
+      </c>
+      <c r="AN57" s="1" t="s">
         <v>575</v>
-      </c>
-      <c r="AN57" s="1" t="s">
-        <v>576</v>
       </c>
       <c r="AO57" s="1"/>
       <c r="AP57" s="1" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="AQ57" s="1" t="s">
         <v>3</v>
@@ -8464,13 +8457,13 @@
     </row>
     <row r="58" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="B58" t="s">
         <v>97</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="D58" t="s">
         <v>27</v>
@@ -8479,10 +8472,10 @@
         <v>28</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="H58" s="1"/>
       <c r="I58" s="1"/>
@@ -8500,7 +8493,7 @@
       <c r="U58" s="1"/>
       <c r="V58" s="1"/>
       <c r="W58" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="X58" s="1"/>
       <c r="Y58" s="1"/>
@@ -8511,32 +8504,32 @@
         <v>44</v>
       </c>
       <c r="AE58" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="AF58">
         <v>1</v>
       </c>
       <c r="AG58" t="s">
+        <v>581</v>
+      </c>
+      <c r="AH58" t="s">
         <v>582</v>
-      </c>
-      <c r="AH58" t="s">
-        <v>583</v>
       </c>
       <c r="AK58" t="s">
         <v>92</v>
       </c>
       <c r="AL58" t="s">
+        <v>583</v>
+      </c>
+      <c r="AM58" s="1" t="s">
         <v>584</v>
       </c>
-      <c r="AM58" s="1" t="s">
+      <c r="AN58" s="1" t="s">
         <v>585</v>
-      </c>
-      <c r="AN58" s="1" t="s">
-        <v>586</v>
       </c>
       <c r="AO58" s="1"/>
       <c r="AP58" s="1" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AQ58" s="1" t="s">
         <v>3</v>
@@ -8544,13 +8537,13 @@
     </row>
     <row r="59" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="B59" t="s">
         <v>97</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="D59" t="s">
         <v>27</v>
@@ -8559,10 +8552,10 @@
         <v>28</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="H59" s="1"/>
       <c r="I59" s="1"/>
@@ -8580,7 +8573,7 @@
       <c r="U59" s="1"/>
       <c r="V59" s="1"/>
       <c r="W59" s="1" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="X59" s="1"/>
       <c r="Y59" s="1"/>
@@ -8612,16 +8605,16 @@
         <v>50</v>
       </c>
       <c r="AM59" s="1" t="s">
+        <v>590</v>
+      </c>
+      <c r="AN59" s="1" t="s">
         <v>591</v>
       </c>
-      <c r="AN59" s="1" t="s">
+      <c r="AO59" s="1" t="s">
         <v>592</v>
       </c>
-      <c r="AO59" s="1" t="s">
+      <c r="AP59" s="1" t="s">
         <v>593</v>
-      </c>
-      <c r="AP59" s="1" t="s">
-        <v>594</v>
       </c>
       <c r="AQ59" s="1" t="s">
         <v>3</v>
@@ -8629,13 +8622,13 @@
     </row>
     <row r="60" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B60" t="s">
         <v>97</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="D60" t="s">
         <v>27</v>
@@ -8644,10 +8637,10 @@
         <v>28</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="H60" s="1"/>
       <c r="I60" s="1"/>
@@ -8665,7 +8658,7 @@
       <c r="U60" s="1"/>
       <c r="V60" s="1"/>
       <c r="W60" s="1" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="X60" s="1"/>
       <c r="Y60" s="1"/>
@@ -8682,7 +8675,7 @@
         <v>1</v>
       </c>
       <c r="AG60" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="AH60" t="s">
         <v>279</v>
@@ -8697,16 +8690,16 @@
         <v>50</v>
       </c>
       <c r="AM60" s="1" t="s">
+        <v>596</v>
+      </c>
+      <c r="AN60" s="1" t="s">
         <v>597</v>
       </c>
-      <c r="AN60" s="1" t="s">
+      <c r="AO60" s="1" t="s">
         <v>598</v>
       </c>
-      <c r="AO60" s="1" t="s">
+      <c r="AP60" s="1" t="s">
         <v>599</v>
-      </c>
-      <c r="AP60" s="1" t="s">
-        <v>600</v>
       </c>
       <c r="AQ60" s="1" t="s">
         <v>3</v>
@@ -8714,13 +8707,13 @@
     </row>
     <row r="61" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B61" t="s">
         <v>97</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="D61" t="s">
         <v>27</v>
@@ -8729,10 +8722,10 @@
         <v>28</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="H61" s="1"/>
       <c r="I61" s="1"/>
@@ -8750,7 +8743,7 @@
       <c r="U61" s="1"/>
       <c r="V61" s="1"/>
       <c r="W61" s="1" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="X61" s="1"/>
       <c r="Y61" s="1"/>
@@ -8779,16 +8772,16 @@
         <v>103</v>
       </c>
       <c r="AM61" s="1" t="s">
+        <v>601</v>
+      </c>
+      <c r="AN61" s="1" t="s">
         <v>602</v>
       </c>
-      <c r="AN61" s="1" t="s">
+      <c r="AO61" s="1" t="s">
         <v>603</v>
       </c>
-      <c r="AO61" s="1" t="s">
+      <c r="AP61" s="1" t="s">
         <v>604</v>
-      </c>
-      <c r="AP61" s="1" t="s">
-        <v>605</v>
       </c>
       <c r="AQ61" s="1" t="s">
         <v>3</v>
@@ -8853,7 +8846,7 @@
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>1</v>
@@ -8868,10 +8861,10 @@
         <v>241</v>
       </c>
       <c r="H1" s="2" t="s">
+        <v>606</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>607</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>608</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>6</v>
@@ -8930,7 +8923,7 @@
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B2" t="s">
         <v>97</v>
@@ -8945,10 +8938,10 @@
         <v>28</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="H2">
         <v>36</v>
@@ -8967,20 +8960,20 @@
       <c r="U2" s="1"/>
       <c r="V2" s="1"/>
       <c r="W2" s="1" t="s">
+        <v>609</v>
+      </c>
+      <c r="X2" s="1" t="s">
         <v>610</v>
-      </c>
-      <c r="X2" s="1" t="s">
-        <v>611</v>
       </c>
       <c r="Y2" s="1"/>
       <c r="Z2" s="1"/>
       <c r="AA2" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="B3" t="s">
         <v>97</v>
@@ -8995,10 +8988,10 @@
         <v>28</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="H3">
         <v>36</v>
@@ -9017,20 +9010,20 @@
       <c r="U3" s="1"/>
       <c r="V3" s="1"/>
       <c r="W3" s="1" t="s">
+        <v>613</v>
+      </c>
+      <c r="X3" s="1" t="s">
         <v>614</v>
-      </c>
-      <c r="X3" s="1" t="s">
-        <v>615</v>
       </c>
       <c r="Y3" s="1"/>
       <c r="Z3" s="1"/>
       <c r="AA3" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="B4" t="s">
         <v>97</v>
@@ -9045,10 +9038,10 @@
         <v>28</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="H4">
         <v>14</v>
@@ -9067,20 +9060,20 @@
       <c r="U4" s="1"/>
       <c r="V4" s="1"/>
       <c r="W4" s="1" t="s">
+        <v>616</v>
+      </c>
+      <c r="X4" s="1" t="s">
         <v>617</v>
-      </c>
-      <c r="X4" s="1" t="s">
-        <v>618</v>
       </c>
       <c r="Y4" s="1"/>
       <c r="Z4" s="1"/>
       <c r="AA4" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="B5" t="s">
         <v>97</v>
@@ -9095,10 +9088,10 @@
         <v>28</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
@@ -9111,20 +9104,20 @@
       <c r="U5" s="1"/>
       <c r="V5" s="1"/>
       <c r="W5" s="1" t="s">
+        <v>619</v>
+      </c>
+      <c r="X5" s="1" t="s">
         <v>620</v>
-      </c>
-      <c r="X5" s="1" t="s">
-        <v>621</v>
       </c>
       <c r="Y5" s="1"/>
       <c r="Z5" s="1"/>
       <c r="AA5" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B6" t="s">
         <v>97</v>
@@ -9139,10 +9132,10 @@
         <v>28</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
@@ -9155,20 +9148,20 @@
       <c r="U6" s="1"/>
       <c r="V6" s="1"/>
       <c r="W6" s="1" t="s">
+        <v>622</v>
+      </c>
+      <c r="X6" s="1" t="s">
         <v>623</v>
-      </c>
-      <c r="X6" s="1" t="s">
-        <v>624</v>
       </c>
       <c r="Y6" s="1"/>
       <c r="Z6" s="1"/>
       <c r="AA6" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B7" t="s">
         <v>97</v>
@@ -9183,10 +9176,10 @@
         <v>28</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
@@ -9199,20 +9192,20 @@
       <c r="U7" s="1"/>
       <c r="V7" s="1"/>
       <c r="W7" s="1" t="s">
+        <v>625</v>
+      </c>
+      <c r="X7" s="1" t="s">
         <v>626</v>
-      </c>
-      <c r="X7" s="1" t="s">
-        <v>627</v>
       </c>
       <c r="Y7" s="1"/>
       <c r="Z7" s="1"/>
       <c r="AA7" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="B8" t="s">
         <v>97</v>
@@ -9227,10 +9220,10 @@
         <v>28</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
@@ -9243,20 +9236,20 @@
       <c r="U8" s="1"/>
       <c r="V8" s="1"/>
       <c r="W8" s="1" t="s">
+        <v>628</v>
+      </c>
+      <c r="X8" s="1" t="s">
         <v>629</v>
-      </c>
-      <c r="X8" s="1" t="s">
-        <v>630</v>
       </c>
       <c r="Y8" s="1"/>
       <c r="Z8" s="1"/>
       <c r="AA8" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B9" t="s">
         <v>97</v>
@@ -9271,10 +9264,10 @@
         <v>28</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="H9">
         <v>16</v>
@@ -9293,20 +9286,20 @@
       <c r="U9" s="1"/>
       <c r="V9" s="1"/>
       <c r="W9" s="1" t="s">
+        <v>631</v>
+      </c>
+      <c r="X9" s="1" t="s">
         <v>632</v>
-      </c>
-      <c r="X9" s="1" t="s">
-        <v>633</v>
       </c>
       <c r="Y9" s="1"/>
       <c r="Z9" s="1"/>
       <c r="AA9" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B10" t="s">
         <v>97</v>
@@ -9321,10 +9314,10 @@
         <v>28</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="H10">
         <v>36</v>
@@ -9343,20 +9336,20 @@
       <c r="U10" s="1"/>
       <c r="V10" s="1"/>
       <c r="W10" s="1" t="s">
+        <v>634</v>
+      </c>
+      <c r="X10" s="1" t="s">
         <v>635</v>
-      </c>
-      <c r="X10" s="1" t="s">
-        <v>636</v>
       </c>
       <c r="Y10" s="1"/>
       <c r="Z10" s="1"/>
       <c r="AA10" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B11" t="s">
         <v>97</v>
@@ -9371,10 +9364,10 @@
         <v>28</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="H11">
         <v>36</v>
@@ -9387,27 +9380,27 @@
       </c>
       <c r="L11" s="1"/>
       <c r="M11" s="1" t="s">
+        <v>637</v>
+      </c>
+      <c r="N11" s="1" t="s">
         <v>638</v>
       </c>
-      <c r="N11" s="1" t="s">
-        <v>639</v>
-      </c>
       <c r="O11" s="1" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="P11" s="1"/>
       <c r="R11" s="1" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="S11" s="1"/>
       <c r="T11" s="1"/>
       <c r="U11" s="1"/>
       <c r="V11" s="1"/>
       <c r="W11" s="1" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="X11" s="1" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="Y11" s="1"/>
       <c r="Z11" s="1"/>
@@ -9417,7 +9410,7 @@
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B12" t="s">
         <v>97</v>
@@ -9432,10 +9425,10 @@
         <v>28</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="H12">
         <v>32</v>
@@ -9448,30 +9441,30 @@
       </c>
       <c r="L12" s="1"/>
       <c r="M12" s="1" t="s">
+        <v>642</v>
+      </c>
+      <c r="N12" s="1" t="s">
         <v>643</v>
       </c>
-      <c r="N12" s="1" t="s">
-        <v>644</v>
-      </c>
       <c r="O12" s="1" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="P12" s="1"/>
       <c r="R12" s="1" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="S12" s="1"/>
       <c r="T12" s="1"/>
       <c r="U12" s="1"/>
       <c r="V12" s="1"/>
       <c r="W12" s="1" t="s">
+        <v>645</v>
+      </c>
+      <c r="X12" s="1" t="s">
         <v>646</v>
       </c>
-      <c r="X12" s="1" t="s">
+      <c r="Y12" s="1" t="s">
         <v>647</v>
-      </c>
-      <c r="Y12" s="1" t="s">
-        <v>648</v>
       </c>
       <c r="Z12" s="1"/>
       <c r="AA12" s="1" t="s">
@@ -9480,7 +9473,7 @@
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B13" t="s">
         <v>97</v>
@@ -9495,16 +9488,16 @@
         <v>28</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="H13">
         <v>48</v>
       </c>
       <c r="I13" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
@@ -9517,20 +9510,20 @@
       <c r="U13" s="1"/>
       <c r="V13" s="1"/>
       <c r="W13" s="1" t="s">
+        <v>650</v>
+      </c>
+      <c r="X13" s="1" t="s">
         <v>651</v>
-      </c>
-      <c r="X13" s="1" t="s">
-        <v>652</v>
       </c>
       <c r="Y13" s="1"/>
       <c r="Z13" s="1"/>
       <c r="AA13" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B14" t="s">
         <v>97</v>
@@ -9545,16 +9538,16 @@
         <v>28</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="H14">
         <v>48</v>
       </c>
       <c r="I14" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
@@ -9567,20 +9560,20 @@
       <c r="U14" s="1"/>
       <c r="V14" s="1"/>
       <c r="W14" s="1" t="s">
+        <v>653</v>
+      </c>
+      <c r="X14" s="1" t="s">
         <v>654</v>
-      </c>
-      <c r="X14" s="1" t="s">
-        <v>655</v>
       </c>
       <c r="Y14" s="1"/>
       <c r="Z14" s="1"/>
       <c r="AA14" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="B15" t="s">
         <v>97</v>
@@ -9595,10 +9588,10 @@
         <v>28</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="H15">
         <v>24</v>
@@ -9617,20 +9610,20 @@
       <c r="U15" s="1"/>
       <c r="V15" s="1"/>
       <c r="W15" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="X15" s="1" t="s">
         <v>657</v>
-      </c>
-      <c r="X15" s="1" t="s">
-        <v>658</v>
       </c>
       <c r="Y15" s="1"/>
       <c r="Z15" s="1"/>
       <c r="AA15" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B16" t="s">
         <v>97</v>
@@ -9645,10 +9638,10 @@
         <v>28</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="H16">
         <v>36</v>
@@ -9667,20 +9660,20 @@
       <c r="U16" s="1"/>
       <c r="V16" s="1"/>
       <c r="W16" s="1" t="s">
+        <v>659</v>
+      </c>
+      <c r="X16" s="1" t="s">
         <v>660</v>
-      </c>
-      <c r="X16" s="1" t="s">
-        <v>661</v>
       </c>
       <c r="Y16" s="1"/>
       <c r="Z16" s="1"/>
       <c r="AA16" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="B17" t="s">
         <v>97</v>
@@ -9695,10 +9688,10 @@
         <v>28</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="H17">
         <v>36</v>
@@ -9717,20 +9710,20 @@
       <c r="U17" s="1"/>
       <c r="V17" s="1"/>
       <c r="W17" s="1" t="s">
+        <v>662</v>
+      </c>
+      <c r="X17" s="1" t="s">
         <v>663</v>
-      </c>
-      <c r="X17" s="1" t="s">
-        <v>664</v>
       </c>
       <c r="Y17" s="1"/>
       <c r="Z17" s="1"/>
       <c r="AA17" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B18" t="s">
         <v>97</v>
@@ -9745,16 +9738,16 @@
         <v>28</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="H18">
         <v>36</v>
       </c>
       <c r="I18" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="L18" s="1"/>
       <c r="M18" s="1"/>
@@ -9767,20 +9760,20 @@
       <c r="U18" s="1"/>
       <c r="V18" s="1"/>
       <c r="W18" s="1" t="s">
+        <v>666</v>
+      </c>
+      <c r="X18" s="1" t="s">
         <v>667</v>
-      </c>
-      <c r="X18" s="1" t="s">
-        <v>668</v>
       </c>
       <c r="Y18" s="1"/>
       <c r="Z18" s="1"/>
       <c r="AA18" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="B19" t="s">
         <v>97</v>
@@ -9795,10 +9788,10 @@
         <v>28</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="H19">
         <v>32</v>
@@ -9817,20 +9810,20 @@
       <c r="U19" s="1"/>
       <c r="V19" s="1"/>
       <c r="W19" s="1" t="s">
+        <v>669</v>
+      </c>
+      <c r="X19" s="1" t="s">
         <v>670</v>
-      </c>
-      <c r="X19" s="1" t="s">
-        <v>671</v>
       </c>
       <c r="Y19" s="1"/>
       <c r="Z19" s="1"/>
       <c r="AA19" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="B20" t="s">
         <v>97</v>
@@ -9845,10 +9838,10 @@
         <v>28</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="L20" s="1"/>
       <c r="M20" s="1"/>
@@ -9861,20 +9854,20 @@
       <c r="U20" s="1"/>
       <c r="V20" s="1"/>
       <c r="W20" s="1" t="s">
+        <v>672</v>
+      </c>
+      <c r="X20" s="1" t="s">
         <v>673</v>
-      </c>
-      <c r="X20" s="1" t="s">
-        <v>674</v>
       </c>
       <c r="Y20" s="1"/>
       <c r="Z20" s="1"/>
       <c r="AA20" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B21" t="s">
         <v>97</v>
@@ -9889,10 +9882,10 @@
         <v>28</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="L21" s="1"/>
       <c r="M21" s="1"/>
@@ -9905,20 +9898,20 @@
       <c r="U21" s="1"/>
       <c r="V21" s="1"/>
       <c r="W21" s="1" t="s">
+        <v>675</v>
+      </c>
+      <c r="X21" s="1" t="s">
         <v>676</v>
-      </c>
-      <c r="X21" s="1" t="s">
-        <v>677</v>
       </c>
       <c r="Y21" s="1"/>
       <c r="Z21" s="1"/>
       <c r="AA21" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="B22" t="s">
         <v>97</v>
@@ -9933,10 +9926,10 @@
         <v>28</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="L22" s="1"/>
       <c r="M22" s="1"/>
@@ -9949,20 +9942,20 @@
       <c r="U22" s="1"/>
       <c r="V22" s="1"/>
       <c r="W22" s="1" t="s">
+        <v>678</v>
+      </c>
+      <c r="X22" s="1" t="s">
         <v>679</v>
-      </c>
-      <c r="X22" s="1" t="s">
-        <v>680</v>
       </c>
       <c r="Y22" s="1"/>
       <c r="Z22" s="1"/>
       <c r="AA22" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="B23" t="s">
         <v>97</v>
@@ -9977,10 +9970,10 @@
         <v>28</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="L23" s="1"/>
       <c r="M23" s="1"/>
@@ -9993,20 +9986,20 @@
       <c r="U23" s="1"/>
       <c r="V23" s="1"/>
       <c r="W23" s="1" t="s">
+        <v>681</v>
+      </c>
+      <c r="X23" s="1" t="s">
         <v>682</v>
-      </c>
-      <c r="X23" s="1" t="s">
-        <v>683</v>
       </c>
       <c r="Y23" s="1"/>
       <c r="Z23" s="1"/>
       <c r="AA23" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="B24" t="s">
         <v>97</v>
@@ -10021,10 +10014,10 @@
         <v>28</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="L24" s="1"/>
       <c r="M24" s="1"/>
@@ -10037,20 +10030,20 @@
       <c r="U24" s="1"/>
       <c r="V24" s="1"/>
       <c r="W24" s="1" t="s">
+        <v>684</v>
+      </c>
+      <c r="X24" s="1" t="s">
         <v>685</v>
-      </c>
-      <c r="X24" s="1" t="s">
-        <v>686</v>
       </c>
       <c r="Y24" s="1"/>
       <c r="Z24" s="1"/>
       <c r="AA24" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="B25" t="s">
         <v>97</v>
@@ -10065,10 +10058,10 @@
         <v>28</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="L25" s="1"/>
       <c r="M25" s="1"/>
@@ -10081,20 +10074,20 @@
       <c r="U25" s="1"/>
       <c r="V25" s="1"/>
       <c r="W25" s="1" t="s">
+        <v>687</v>
+      </c>
+      <c r="X25" s="1" t="s">
         <v>688</v>
-      </c>
-      <c r="X25" s="1" t="s">
-        <v>689</v>
       </c>
       <c r="Y25" s="1"/>
       <c r="Z25" s="1"/>
       <c r="AA25" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="B26" t="s">
         <v>97</v>
@@ -10109,10 +10102,10 @@
         <v>28</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
@@ -10125,20 +10118,20 @@
       <c r="U26" s="1"/>
       <c r="V26" s="1"/>
       <c r="W26" s="1" t="s">
+        <v>690</v>
+      </c>
+      <c r="X26" s="1" t="s">
         <v>691</v>
-      </c>
-      <c r="X26" s="1" t="s">
-        <v>692</v>
       </c>
       <c r="Y26" s="1"/>
       <c r="Z26" s="1"/>
       <c r="AA26" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="27" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="B27" t="s">
         <v>97</v>
@@ -10153,10 +10146,10 @@
         <v>28</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
@@ -10169,20 +10162,20 @@
       <c r="U27" s="1"/>
       <c r="V27" s="1"/>
       <c r="W27" s="1" t="s">
+        <v>693</v>
+      </c>
+      <c r="X27" s="1" t="s">
         <v>694</v>
-      </c>
-      <c r="X27" s="1" t="s">
-        <v>695</v>
       </c>
       <c r="Y27" s="1"/>
       <c r="Z27" s="1"/>
       <c r="AA27" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="28" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="B28" t="s">
         <v>97</v>
@@ -10197,10 +10190,10 @@
         <v>28</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
@@ -10213,20 +10206,20 @@
       <c r="U28" s="1"/>
       <c r="V28" s="1"/>
       <c r="W28" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="X28" s="1" t="s">
         <v>697</v>
-      </c>
-      <c r="X28" s="1" t="s">
-        <v>698</v>
       </c>
       <c r="Y28" s="1"/>
       <c r="Z28" s="1"/>
       <c r="AA28" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="29" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="B29" t="s">
         <v>97</v>
@@ -10241,10 +10234,10 @@
         <v>28</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
@@ -10257,20 +10250,20 @@
       <c r="U29" s="1"/>
       <c r="V29" s="1"/>
       <c r="W29" s="1" t="s">
+        <v>699</v>
+      </c>
+      <c r="X29" s="1" t="s">
         <v>700</v>
-      </c>
-      <c r="X29" s="1" t="s">
-        <v>701</v>
       </c>
       <c r="Y29" s="1"/>
       <c r="Z29" s="1"/>
       <c r="AA29" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="30" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="B30" t="s">
         <v>97</v>
@@ -10285,10 +10278,10 @@
         <v>28</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="H30">
         <v>8</v>
@@ -10307,20 +10300,20 @@
       <c r="U30" s="1"/>
       <c r="V30" s="1"/>
       <c r="W30" s="1" t="s">
+        <v>702</v>
+      </c>
+      <c r="X30" s="1" t="s">
         <v>703</v>
-      </c>
-      <c r="X30" s="1" t="s">
-        <v>704</v>
       </c>
       <c r="Y30" s="1"/>
       <c r="Z30" s="1"/>
       <c r="AA30" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="31" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="B31" t="s">
         <v>97</v>
@@ -10335,16 +10328,16 @@
         <v>28</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="H31">
         <v>16</v>
       </c>
       <c r="I31" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
@@ -10357,20 +10350,20 @@
       <c r="U31" s="1"/>
       <c r="V31" s="1"/>
       <c r="W31" s="1" t="s">
+        <v>706</v>
+      </c>
+      <c r="X31" s="1" t="s">
         <v>707</v>
-      </c>
-      <c r="X31" s="1" t="s">
-        <v>708</v>
       </c>
       <c r="Y31" s="1"/>
       <c r="Z31" s="1"/>
       <c r="AA31" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="32" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="B32" t="s">
         <v>97</v>
@@ -10385,16 +10378,16 @@
         <v>28</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="H32">
         <v>22</v>
       </c>
       <c r="I32" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
@@ -10407,20 +10400,20 @@
       <c r="U32" s="1"/>
       <c r="V32" s="1"/>
       <c r="W32" s="1" t="s">
+        <v>710</v>
+      </c>
+      <c r="X32" s="1" t="s">
         <v>711</v>
-      </c>
-      <c r="X32" s="1" t="s">
-        <v>712</v>
       </c>
       <c r="Y32" s="1"/>
       <c r="Z32" s="1"/>
       <c r="AA32" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="33" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="B33" t="s">
         <v>97</v>
@@ -10435,16 +10428,16 @@
         <v>28</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="H33">
         <v>24</v>
       </c>
       <c r="I33" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="L33" s="1"/>
       <c r="M33" s="1"/>
@@ -10457,20 +10450,20 @@
       <c r="U33" s="1"/>
       <c r="V33" s="1"/>
       <c r="W33" s="1" t="s">
+        <v>714</v>
+      </c>
+      <c r="X33" s="1" t="s">
         <v>715</v>
-      </c>
-      <c r="X33" s="1" t="s">
-        <v>716</v>
       </c>
       <c r="Y33" s="1"/>
       <c r="Z33" s="1"/>
       <c r="AA33" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="34" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="B34" t="s">
         <v>97</v>
@@ -10485,16 +10478,16 @@
         <v>28</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="H34">
         <v>48</v>
       </c>
       <c r="I34" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="L34" s="1"/>
       <c r="M34" s="1"/>
@@ -10507,20 +10500,20 @@
       <c r="U34" s="1"/>
       <c r="V34" s="1"/>
       <c r="W34" s="1" t="s">
+        <v>717</v>
+      </c>
+      <c r="X34" s="1" t="s">
         <v>718</v>
-      </c>
-      <c r="X34" s="1" t="s">
-        <v>719</v>
       </c>
       <c r="Y34" s="1"/>
       <c r="Z34" s="1"/>
       <c r="AA34" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="35" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="B35" t="s">
         <v>97</v>
@@ -10535,16 +10528,16 @@
         <v>28</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="H35">
         <v>48</v>
       </c>
       <c r="I35" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="L35" s="1"/>
       <c r="M35" s="1"/>
@@ -10557,20 +10550,20 @@
       <c r="U35" s="1"/>
       <c r="V35" s="1"/>
       <c r="W35" s="1" t="s">
+        <v>720</v>
+      </c>
+      <c r="X35" s="1" t="s">
         <v>721</v>
-      </c>
-      <c r="X35" s="1" t="s">
-        <v>722</v>
       </c>
       <c r="Y35" s="1"/>
       <c r="Z35" s="1"/>
       <c r="AA35" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="36" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="B36" t="s">
         <v>97</v>
@@ -10585,16 +10578,16 @@
         <v>28</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="H36">
         <v>48</v>
       </c>
       <c r="I36" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
@@ -10607,20 +10600,20 @@
       <c r="U36" s="1"/>
       <c r="V36" s="1"/>
       <c r="W36" s="1" t="s">
+        <v>723</v>
+      </c>
+      <c r="X36" s="1" t="s">
         <v>724</v>
-      </c>
-      <c r="X36" s="1" t="s">
-        <v>725</v>
       </c>
       <c r="Y36" s="1"/>
       <c r="Z36" s="1"/>
       <c r="AA36" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="37" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="B37" t="s">
         <v>97</v>
@@ -10635,16 +10628,16 @@
         <v>28</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="H37">
         <v>48</v>
       </c>
       <c r="I37" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="L37" s="1"/>
       <c r="M37" s="1"/>
@@ -10657,20 +10650,20 @@
       <c r="U37" s="1"/>
       <c r="V37" s="1"/>
       <c r="W37" s="1" t="s">
+        <v>726</v>
+      </c>
+      <c r="X37" s="1" t="s">
         <v>727</v>
-      </c>
-      <c r="X37" s="1" t="s">
-        <v>728</v>
       </c>
       <c r="Y37" s="1"/>
       <c r="Z37" s="1"/>
       <c r="AA37" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="38" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="B38" t="s">
         <v>97</v>
@@ -10685,10 +10678,10 @@
         <v>28</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="L38" s="1"/>
       <c r="M38" s="1"/>
@@ -10701,20 +10694,20 @@
       <c r="U38" s="1"/>
       <c r="V38" s="1"/>
       <c r="W38" s="1" t="s">
+        <v>729</v>
+      </c>
+      <c r="X38" s="1" t="s">
         <v>730</v>
-      </c>
-      <c r="X38" s="1" t="s">
-        <v>731</v>
       </c>
       <c r="Y38" s="1"/>
       <c r="Z38" s="1"/>
       <c r="AA38" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="39" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="B39" t="s">
         <v>97</v>
@@ -10729,10 +10722,10 @@
         <v>28</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="L39" s="1"/>
       <c r="M39" s="1"/>
@@ -10745,20 +10738,20 @@
       <c r="U39" s="1"/>
       <c r="V39" s="1"/>
       <c r="W39" s="1" t="s">
+        <v>732</v>
+      </c>
+      <c r="X39" s="1" t="s">
         <v>733</v>
-      </c>
-      <c r="X39" s="1" t="s">
-        <v>734</v>
       </c>
       <c r="Y39" s="1"/>
       <c r="Z39" s="1"/>
       <c r="AA39" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="40" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="B40" t="s">
         <v>97</v>
@@ -10773,10 +10766,10 @@
         <v>28</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="L40" s="1"/>
       <c r="M40" s="1"/>
@@ -10789,15 +10782,15 @@
       <c r="U40" s="1"/>
       <c r="V40" s="1"/>
       <c r="W40" s="1" t="s">
+        <v>735</v>
+      </c>
+      <c r="X40" s="1" t="s">
         <v>736</v>
-      </c>
-      <c r="X40" s="1" t="s">
-        <v>737</v>
       </c>
       <c r="Y40" s="1"/>
       <c r="Z40" s="1"/>
       <c r="AA40" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
   </sheetData>
@@ -10838,827 +10831,827 @@
   <sheetData>
     <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>737</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>738</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>739</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>740</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>274</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>284</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>274</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>284</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>274</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>284</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>274</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>284</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>274</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>284</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>274</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>284</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>274</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>284</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>287</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>287</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>299</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>287</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>299</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>287</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>299</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>287</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>299</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>287</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>299</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>287</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>287</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>287</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>287</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>287</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>287</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>287</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>299</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>287</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>299</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>287</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="B54" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="B55" s="1" t="s">
         <v>299</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="B56" s="1" t="s">
         <v>302</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="B57" s="1" t="s">
         <v>302</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="B58" s="1" t="s">
         <v>302</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
     </row>
   </sheetData>
@@ -11693,10 +11686,10 @@
         <v>2</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>753</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>754</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>755</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -11704,7 +11697,7 @@
         <v>97</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="C2" t="s">
         <v>27</v>
@@ -11720,7 +11713,7 @@
         <v>97</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="C3" t="s">
         <v>27</v>
@@ -11736,7 +11729,7 @@
         <v>97</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="C4" t="s">
         <v>27</v>
@@ -11752,7 +11745,7 @@
         <v>97</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C5" t="s">
         <v>27</v>
@@ -12024,7 +12017,7 @@
         <v>97</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="C22" t="s">
         <v>27</v>

</xml_diff>